<commit_message>
f29h85x : CDD IPC, CDD UART : Generate Test Report for C29xMCAL_01.02.01.06
- Generate Test Report for C29xMCAL_01.02.01.06

Fixes: MCAL-30841

Signed-off-by: Piyush Panditrao <p-panditrao@ti.com>
</commit_message>
<xml_diff>
--- a/docs/Test_Report/Cdd_Uart/TestPlanExecutionReport_Cdd_Uart.xlsx
+++ b/docs/Test_Report/Cdd_Uart/TestPlanExecutionReport_Cdd_Uart.xlsx
@@ -43,7 +43,7 @@
       <sz val="16"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -77,11 +77,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000000FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
@@ -104,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -136,13 +131,10 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -734,7 +726,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2025-06-09 06:51:21.839842-05:00 CDT</t>
+          <t>2025-06-10 02:10:58.413311-05:00 CDT</t>
         </is>
       </c>
     </row>
@@ -806,12 +798,12 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>48</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -1028,12 +1020,12 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>58</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1119,12 +1111,12 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>17%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>83%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -6226,9 +6218,9 @@
       </c>
       <c r="S52" s="3" t="inlineStr"/>
       <c r="T52" s="3" t="inlineStr"/>
-      <c r="U52" s="11" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+      <c r="U52" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -6317,9 +6309,9 @@
       </c>
       <c r="S53" s="3" t="inlineStr"/>
       <c r="T53" s="3" t="inlineStr"/>
-      <c r="U53" s="11" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+      <c r="U53" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -6408,9 +6400,9 @@
       </c>
       <c r="S54" s="3" t="inlineStr"/>
       <c r="T54" s="3" t="inlineStr"/>
-      <c r="U54" s="11" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+      <c r="U54" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -6503,9 +6495,9 @@
       </c>
       <c r="S55" s="3" t="inlineStr"/>
       <c r="T55" s="3" t="inlineStr"/>
-      <c r="U55" s="11" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+      <c r="U55" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -6594,9 +6586,9 @@
       </c>
       <c r="S56" s="3" t="inlineStr"/>
       <c r="T56" s="3" t="inlineStr"/>
-      <c r="U56" s="11" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+      <c r="U56" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -6685,9 +6677,9 @@
       </c>
       <c r="S57" s="3" t="inlineStr"/>
       <c r="T57" s="3" t="inlineStr"/>
-      <c r="U57" s="11" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+      <c r="U57" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -6780,9 +6772,9 @@
       </c>
       <c r="S58" s="3" t="inlineStr"/>
       <c r="T58" s="3" t="inlineStr"/>
-      <c r="U58" s="11" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+      <c r="U58" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -6871,9 +6863,9 @@
       </c>
       <c r="S59" s="3" t="inlineStr"/>
       <c r="T59" s="3" t="inlineStr"/>
-      <c r="U59" s="11" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+      <c r="U59" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -6927,12 +6919,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Test Plan</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>Test Plan Key</t>
         </is>
@@ -6954,8 +6946,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="n"/>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="A3" s="11" t="n"/>
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Test Plan Name</t>
         </is>
@@ -6977,8 +6969,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="n"/>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="A4" s="11" t="n"/>
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Test Case Key</t>
         </is>
@@ -7000,8 +6992,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="n"/>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="A5" s="11" t="n"/>
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Test Case Name</t>
         </is>
@@ -7023,8 +7015,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n"/>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Associated Issue(s) Type</t>
         </is>
@@ -7051,8 +7043,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="n"/>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Associated Issue(s) ID(s)</t>
         </is>
@@ -7074,8 +7066,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n"/>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Test Platform</t>
         </is>
@@ -7097,8 +7089,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n"/>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Test Level</t>
         </is>
@@ -7114,7 +7106,7 @@
 -- "Not Provided" if no 'Test Scope' is provided in Jira</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7126,8 +7118,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n"/>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Test Description</t>
         </is>
@@ -7149,8 +7141,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="n"/>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Test Setup</t>
         </is>
@@ -7172,8 +7164,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Pass/Fail Criteria</t>
         </is>
@@ -7195,8 +7187,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="n"/>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Test Type</t>
         </is>
@@ -7207,7 +7199,7 @@
 (Map Test Method from Qmetry)</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7219,15 +7211,15 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n"/>
-      <c r="B14" s="13" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="12" t="n"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Functional:
 Tests covering functional requirements-based  aspects of the software</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7239,8 +7231,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="n"/>
-      <c r="B15" s="13" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="12" t="n"/>
       <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Compatability:
@@ -7248,7 +7240,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of testing that measures the degree to which a test item can function satisfactorily alongside other independent products in a shared environment (co-existence), and where necessary, exchanges information with other systems or components (interoperability)</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7260,15 +7252,15 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n"/>
-      <c r="B16" s="13" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="12" t="n"/>
       <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Usability:
 Test Case covers usability/api/look and feel aspects of the module including out-of box (OOB) experience</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7280,15 +7272,15 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="n"/>
-      <c r="B17" s="13" t="n"/>
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="12" t="n"/>
       <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Fault Injection:
 Testing based on injection of errors or faults to ensure no unintended consequences</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7300,8 +7292,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n"/>
-      <c r="B18" s="13" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="12" t="n"/>
       <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Performance: 
@@ -7309,7 +7301,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of testing conducted to evaluate the degree to which a test item accomplishes its designated functions within given constraints of time and other resources</t>
         </is>
       </c>
-      <c r="D18" s="12" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7321,8 +7313,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="n"/>
-      <c r="B19" s="13" t="n"/>
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="12" t="n"/>
       <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Reliability: 
@@ -7330,7 +7322,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of testing conducted to evaluate the ability of a test item to perform its required functions, including evaluating the frequency with which failures occur, when it is used under stated conditions for a specified period of time</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr">
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7342,8 +7334,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="n"/>
-      <c r="B20" s="13" t="n"/>
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="12" t="n"/>
       <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Stress:
@@ -7351,7 +7343,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of performance efficiency testing conducted to evaluate a test item's behaviour under conditions of loading above anticipated or specified capacity requirements, or of resource availability below minimum specified requirements</t>
         </is>
       </c>
-      <c r="D20" s="12" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7363,8 +7355,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="n"/>
-      <c r="B21" s="13" t="n"/>
+      <c r="A21" s="11" t="n"/>
+      <c r="B21" s="12" t="n"/>
       <c r="C21" s="3" t="inlineStr">
         <is>
           <t>Security:
@@ -7372,7 +7364,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of testing conducted to evaluate the degree to which a test item, and associated data and information, are protected so that unauthorized persons or systems cannot use, read, or modify them, and authorized persons or systems are not denied access to them</t>
         </is>
       </c>
-      <c r="D21" s="12" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7384,8 +7376,8 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="n"/>
-      <c r="B22" s="13" t="n"/>
+      <c r="A22" s="11" t="n"/>
+      <c r="B22" s="12" t="n"/>
       <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Maintainability:
@@ -7393,7 +7385,7 @@
 ISO/IEC/IEEE 29119-1 Defn: test type conducted to evaluate the degree of effectiveness and efficiency with which a test item may be modified</t>
         </is>
       </c>
-      <c r="D22" s="12" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7405,8 +7397,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="n"/>
-      <c r="B23" s="13" t="n"/>
+      <c r="A23" s="11" t="n"/>
+      <c r="B23" s="12" t="n"/>
       <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Portability:
@@ -7414,7 +7406,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of testing conducted to evaluate the ease with which a test item can be transferred from one hardware or software environment to another, including the level of modification needed for it to be executed in various types of environment</t>
         </is>
       </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="D23" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7426,8 +7418,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="n"/>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="A24" s="11" t="n"/>
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>Test Design Technique</t>
         </is>
@@ -7439,7 +7431,7 @@
 (Map Test Derivation Method from Qmetry)</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7451,8 +7443,8 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="n"/>
-      <c r="B25" s="13" t="n"/>
+      <c r="A25" s="11" t="n"/>
+      <c r="B25" s="12" t="n"/>
       <c r="C25" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Requirements-Analysis:
@@ -7460,7 +7452,7 @@
 </t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7472,15 +7464,15 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="n"/>
-      <c r="B26" s="13" t="n"/>
+      <c r="A26" s="11" t="n"/>
+      <c r="B26" s="12" t="n"/>
       <c r="C26" s="3" t="inlineStr">
         <is>
           <t>Boundary Value Analysis:
 Test cases that apply to interfaces and values approaching and crossing the boundaries and out of range values</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7492,15 +7484,15 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="n"/>
-      <c r="B27" s="13" t="n"/>
+      <c r="A27" s="11" t="n"/>
+      <c r="B27" s="12" t="n"/>
       <c r="C27" s="3" t="inlineStr">
         <is>
           <t>Error Guessing:
 Test cases established based on lessons learned and expert judgement to determine situations that may cause software failures or errors to appear</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="D27" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7512,28 +7504,28 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="n"/>
-      <c r="B28" s="13" t="n"/>
+      <c r="A28" s="11" t="n"/>
+      <c r="B28" s="12" t="n"/>
       <c r="C28" s="3" t="inlineStr">
         <is>
           <t>Other (Use case analysis; Customer Usage; Requirement analysis; Failure Mode analysis):
 Teams are encouraged to use techniques defined by standards such as ISO/IEC/IEEE 29119-4; which needs to be refelcted within Qmetry</t>
         </is>
       </c>
-      <c r="D28" s="12" t="inlineStr">
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="n"/>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="A29" s="11" t="n"/>
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>Test Execution Type</t>
         </is>
@@ -7543,7 +7535,7 @@
           <t>Identifies whether the case is automated or manually or Semi-Automated executed</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="D29" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7555,8 +7547,8 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="n"/>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="A30" s="11" t="n"/>
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>Test Category</t>
         </is>
@@ -7566,7 +7558,7 @@
           <t>Test Categories represent sets of tests that are commonly used.</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr">
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7578,15 +7570,15 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="n"/>
-      <c r="B31" s="13" t="n"/>
+      <c r="A31" s="11" t="n"/>
+      <c r="B31" s="12" t="n"/>
       <c r="C31" s="3" t="inlineStr">
         <is>
           <t>Sanity:
 This Test case is identified to run for Sanity Checks. These are mainly the basic tests that need to be run as part of entry to validate phase</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr">
+      <c r="D31" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7598,15 +7590,15 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="n"/>
-      <c r="B32" s="13" t="n"/>
+      <c r="A32" s="11" t="n"/>
+      <c r="B32" s="12" t="n"/>
       <c r="C32" s="3" t="inlineStr">
         <is>
           <t>Full:
 This category means running all test cases for identified releases</t>
         </is>
       </c>
-      <c r="D32" s="12" t="inlineStr">
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7618,15 +7610,15 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="12" t="n"/>
-      <c r="B33" s="13" t="n"/>
+      <c r="A33" s="11" t="n"/>
+      <c r="B33" s="12" t="n"/>
       <c r="C33" s="3" t="inlineStr">
         <is>
           <t>Base Regression:
 This Test case is identified to run for the Base Regression / maintenance releases</t>
         </is>
       </c>
-      <c r="D33" s="12" t="inlineStr">
+      <c r="D33" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -7638,8 +7630,8 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="12" t="n"/>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="A34" s="11" t="n"/>
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Test Component(s)</t>
         </is>
@@ -7649,24 +7641,24 @@
           <t xml:space="preserve">The field provides the Component(s) (in Jira) to which the Test Case is mapped to. </t>
         </is>
       </c>
-      <c r="D34" s="12" t="inlineStr">
+      <c r="D34" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="E34" s="12" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="14" t="inlineStr">
+      <c r="A35" s="13" t="inlineStr">
         <is>
           <t>Test Execution</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>Build/Release Key</t>
         </is>
@@ -7688,8 +7680,8 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="14" t="n"/>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="A36" s="13" t="n"/>
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>Defect Key</t>
         </is>
@@ -7711,8 +7703,8 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="14" t="n"/>
-      <c r="B37" s="13" t="inlineStr">
+      <c r="A37" s="13" t="n"/>
+      <c r="B37" s="12" t="inlineStr">
         <is>
           <t>Defect Summary</t>
         </is>
@@ -7734,8 +7726,8 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="14" t="n"/>
-      <c r="B38" s="13" t="inlineStr">
+      <c r="A38" s="13" t="n"/>
+      <c r="B38" s="12" t="inlineStr">
         <is>
           <t>Overall Status</t>
         </is>
@@ -7758,8 +7750,8 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="14" t="n"/>
-      <c r="B39" s="13" t="n"/>
+      <c r="A39" s="13" t="n"/>
+      <c r="B39" s="12" t="n"/>
       <c r="C39" s="3" t="inlineStr">
         <is>
           <t>PASS
@@ -7778,8 +7770,8 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="14" t="n"/>
-      <c r="B40" s="13" t="n"/>
+      <c r="A40" s="13" t="n"/>
+      <c r="B40" s="12" t="n"/>
       <c r="C40" s="3" t="inlineStr">
         <is>
           <t>FAIL
@@ -7798,8 +7790,8 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="14" t="n"/>
-      <c r="B41" s="13" t="n"/>
+      <c r="A41" s="13" t="n"/>
+      <c r="B41" s="12" t="n"/>
       <c r="C41" s="3" t="inlineStr">
         <is>
           <t>BLOCKED
@@ -7818,8 +7810,8 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="14" t="n"/>
-      <c r="B42" s="13" t="n"/>
+      <c r="A42" s="13" t="n"/>
+      <c r="B42" s="12" t="n"/>
       <c r="C42" s="3" t="inlineStr">
         <is>
           <t>WIP

</xml_diff>